<commit_message>
Initial commit 3Lab, simple input/output
</commit_message>
<xml_diff>
--- a/2 Reelection/PSP.xlsx
+++ b/2 Reelection/PSP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Medion\Desktop\ADS\2 Reelection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D3BAA24-E84A-4B73-9462-AAA564C153E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAD97F8-5EB5-4C84-8054-63AF2A8487E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LFF" sheetId="1" r:id="rId1"/>
@@ -18,18 +18,137 @@
     <sheet name="DTS" sheetId="3" r:id="rId3"/>
     <sheet name="DFF" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+  <si>
+    <t>Nr</t>
+  </si>
+  <si>
+    <t>Tikrinami punktai</t>
+  </si>
+  <si>
+    <t>Rasta defektų</t>
+  </si>
+  <si>
+    <t>Komentarai</t>
+  </si>
+  <si>
+    <t>Iš viso:</t>
+  </si>
+  <si>
+    <t>Defekto tipas</t>
+  </si>
+  <si>
+    <t>Injekcijos faze</t>
+  </si>
+  <si>
+    <t>Aptikimo faze</t>
+  </si>
+  <si>
+    <t>Kiekis</t>
+  </si>
+  <si>
+    <t>% nuo visų</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Tipas</t>
+  </si>
+  <si>
+    <t>Injekcijos fazė</t>
+  </si>
+  <si>
+    <t>Aptikimo fazė</t>
+  </si>
+  <si>
+    <t>Aptikimo laikas (min)</t>
+  </si>
+  <si>
+    <t>Taisymo laikas (min)</t>
+  </si>
+  <si>
+    <t>Aprašymas</t>
+  </si>
+  <si>
+    <t>Nuo</t>
+  </si>
+  <si>
+    <t>Iki</t>
+  </si>
+  <si>
+    <t>Trukdžiai</t>
+  </si>
+  <si>
+    <t>Laikas</t>
+  </si>
+  <si>
+    <t>Veikla</t>
+  </si>
+  <si>
+    <t>Skaitymas</t>
+  </si>
+  <si>
+    <t>Užduoties ir reikalavimų skaitymas</t>
+  </si>
+  <si>
+    <t>Planavimas</t>
+  </si>
+  <si>
+    <t>Struktūrų sudarymas</t>
+  </si>
+  <si>
+    <t>Programavimas</t>
+  </si>
+  <si>
+    <t>Užbaigiama logika ir kuriami Go.cmd ir makefile su testais</t>
+  </si>
+  <si>
+    <t>Testavimas</t>
+  </si>
+  <si>
+    <t>Minimalus pataisymai</t>
+  </si>
+  <si>
+    <t>PSP veikla</t>
+  </si>
+  <si>
+    <t>Pagrindinė backtrack logika.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reelection.h ir main.c. </t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="177" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-ru-UA,1]hh:mm;@"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -37,16 +156,63 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -54,15 +220,431 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{5EEC9441-955F-43CB-AA4C-96DB16C2CFD9}"/>
+    <cellStyle name="Normal 2 2" xfId="2" xr:uid="{1BD68AC8-CAA7-4F4B-B84E-3900D3C3FC5C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -340,36 +922,451 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.21875" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="42.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18.600000000000001" customHeight="1" thickBot="1">
+      <c r="A1" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="48" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="48" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A2" s="47">
+        <v>46107</v>
+      </c>
+      <c r="B2" s="53">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C2" s="53">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D2" s="53">
+        <v>0</v>
+      </c>
+      <c r="E2" s="53">
+        <f>C2-B2-D2</f>
+        <v>2.0833333333333259E-2</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="49" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A3" s="47">
+        <v>46107</v>
+      </c>
+      <c r="B3" s="53">
+        <v>0.73958333333333337</v>
+      </c>
+      <c r="C3" s="53">
+        <v>0.76041666666666663</v>
+      </c>
+      <c r="D3" s="53">
+        <v>0</v>
+      </c>
+      <c r="E3" s="53">
+        <f t="shared" ref="E3:E8" si="0">C3-B3-D3</f>
+        <v>2.0833333333333259E-2</v>
+      </c>
+      <c r="F3" s="49" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="49" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A4" s="47">
+        <v>46109</v>
+      </c>
+      <c r="B4" s="53">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C4" s="53">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="53">
+        <v>0</v>
+      </c>
+      <c r="E4" s="53">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666685E-2</v>
+      </c>
+      <c r="F4" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="49" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A5" s="47">
+        <v>46110</v>
+      </c>
+      <c r="B5" s="53">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C5" s="53">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D5" s="53">
+        <v>0</v>
+      </c>
+      <c r="E5" s="53">
+        <f>C5-B5-D5</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="F5" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="49" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A6" s="47">
+        <v>46110</v>
+      </c>
+      <c r="B6" s="53">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C6" s="53">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="D6" s="53">
+        <v>0</v>
+      </c>
+      <c r="E6" s="53">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666741E-2</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="49" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A7" s="47">
+        <v>46111</v>
+      </c>
+      <c r="B7" s="53">
+        <v>0.6875</v>
+      </c>
+      <c r="C7" s="53">
+        <v>0.75</v>
+      </c>
+      <c r="D7" s="53">
+        <v>0</v>
+      </c>
+      <c r="E7" s="53">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="F7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="51" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="42" customHeight="1" thickBot="1">
+      <c r="A8" s="47">
+        <v>46111</v>
+      </c>
+      <c r="B8" s="53">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C8" s="53">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="D8" s="53">
+        <v>0</v>
+      </c>
+      <c r="E8" s="53">
+        <f t="shared" si="0"/>
+        <v>1.0416666666666741E-2</v>
+      </c>
+      <c r="F8" s="49" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="50"/>
+    </row>
+    <row r="9" spans="1:7" ht="36.6" customHeight="1"/>
+    <row r="10" spans="1:7" ht="36.6" customHeight="1"/>
+    <row r="11" spans="1:7" ht="36.6" customHeight="1"/>
+    <row r="12" spans="1:7">
+      <c r="E12" s="46"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0AA1DD5-7104-4056-8B3C-6B9EAC02401E}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="4" width="20.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="34.200000000000003" customHeight="1" thickBot="1">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" spans="1:4" ht="34.200000000000003" customHeight="1">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" spans="1:4" ht="34.200000000000003" customHeight="1" thickBot="1">
+      <c r="A10" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="9"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F893FC2-82E7-4054-B487-4F95C351F397}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="5" width="17.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="35.4" customHeight="1" thickBot="1">
+      <c r="A1" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="35.4" customHeight="1">
+      <c r="A2" s="17"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="15"/>
+    </row>
+    <row r="3" spans="1:5" ht="35.4" customHeight="1">
+      <c r="A3" s="18"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="1:5" ht="35.4" customHeight="1" thickBot="1">
+      <c r="A4" s="26"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="16"/>
+    </row>
+    <row r="5" spans="1:5" ht="35.4" customHeight="1" thickBot="1">
+      <c r="A5" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="20"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5EB84BA-02FE-41A0-BFF7-129D48DD4B65}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="8" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="37.200000000000003" customHeight="1" thickBot="1">
+      <c r="A1" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="37" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="37.200000000000003" customHeight="1">
+      <c r="A2" s="34">
+        <v>1</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="32"/>
+    </row>
+    <row r="3" spans="1:8" ht="37.200000000000003" customHeight="1">
+      <c r="A3" s="35">
+        <v>2</v>
+      </c>
+      <c r="B3" s="31"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="33"/>
+    </row>
+    <row r="4" spans="1:8" ht="37.200000000000003" customHeight="1" thickBot="1">
+      <c r="A4" s="39">
+        <v>3</v>
+      </c>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>